<commit_message>
fab(rev5): explode BOM to one row per designator (JLCPCB matcher fix)
JLCPCB failed the upload: BOM designators were ';'-joined strings
('U5;U6', 'D1;D2;...') which don't match the per-designator CPL rows -
'U5,U6,...,U3,U4 don't exist in the BOM' + every ';' string 'doesn't exist
in the CPL'.

Now: BOM has exactly the 82 CPL designators, one per row (csv + xlsx rebuilt;
BOM set == CPL set, verified). User-fitted parts are intentionally absent
from BOTH: the 12 board-mounted toggles (MTS-102/103-M), spare pull-ups
R17/R18, and the optional J5 debug header. Same 82-row BOM regenerated for
the macrofab/ package. README documents the 1:1 match and the user-fitted
list. Zips rebuilt.
</commit_message>
<xml_diff>
--- a/hardware/fab-rev5/imspi8080-rev5-bom.xlsx
+++ b/hardware/fab-rev5/imspi8080-rev5-bom.xlsx
@@ -417,13 +417,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
@@ -564,7 +564,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>U3;U4</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -591,49 +591,49 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>74HC165 PISO shift reg</t>
+          <t>TLC5947 24ch LED driver</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>U5;U6</t>
+          <t>U4</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TSSOP-16</t>
+          <t>HTSSOP-32</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SN74HC165PWR</t>
+          <t>TLC5947DAP</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Switch inputs, daisy-chained.</t>
+          <t>LED drivers, daisy-chained. Extended part (1 line = both).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>microSD socket push-pull</t>
+          <t>74HC165 PISO shift reg</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>U7</t>
+          <t>U5</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SMD push-pull</t>
+          <t>TSSOP-16</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -643,29 +643,29 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>microSD TF push-pull</t>
+          <t>SN74HC165PWR</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Data storage (optional). Pick a JLCPCB-library SMD socket.</t>
+          <t>Switch inputs, daisy-chained.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AMS1117-3.3</t>
+          <t>74HC165 PISO shift reg</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>U8</t>
+          <t>U6</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>SOT-223</t>
+          <t>TSSOP-16</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -675,29 +675,29 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>AMS1117-3.3</t>
+          <t>SN74HC165PWR</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>3.3V logic rail from USB-C #1 VBUS. Basic.</t>
+          <t>Switch inputs, daisy-chained.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AMS1117-3.3</t>
+          <t>microSD socket push-pull</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>U9</t>
+          <t>U7</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>SOT-223</t>
+          <t>SMD push-pull</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -707,29 +707,29 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>AMS1117-3.3</t>
+          <t>microSD TF push-pull</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>3.3V LED anode rail from USB-C #2 VBUS (keeps drivers cool).</t>
+          <t>Data storage (optional). Pick a JLCPCB-library SMD socket.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>USB-C receptacle 16P</t>
+          <t>AMS1117-3.3</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>U8</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>USB-C 16P SMD</t>
+          <t>SOT-223</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -739,29 +739,29 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>AMS1117-3.3</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Power + data to the Pi. 2x CC resistors + 2x D series R.</t>
+          <t>3.3V logic rail from USB-C #1 VBUS. Basic.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>USB-C receptacle 16P</t>
+          <t>AMS1117-3.3</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>U9</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>USB-C 16P SMD</t>
+          <t>SOT-223</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -771,93 +771,93 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>TYPE-C-31-M-12</t>
+          <t>AMS1117-3.3</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Dedicated LED power only (VBUS+GND+CC). No data lines.</t>
+          <t>3.3V LED anode rail from USB-C #2 VBUS (keeps drivers cool).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mini-toggle SPDT ON-ON (latching)</t>
+          <t>USB-C receptacle 16P</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SWD0;SWD1;SWD2;SWD3;SWD4;SWD5;SWD6;SWD7</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MTS-102</t>
+          <t>USB-C 16P SMD</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>MTS-102</t>
+          <t>TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>8 latching data toggles (D7..D0), board-mounted, bushing through PCB void</t>
+          <t>Power + data to the Pi. 2x CC resistors + 2x D series R.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Mini-toggle SPDT momentary"</t>
+          <t>USB-C receptacle 16P</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SWC0;SWC1;SWC2;SWC3</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MTS-103-M</t>
+          <t>USB-C 16P SMD</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>MTS-103-M</t>
+          <t>TYPE-C-31-M-12</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>4 momentary command toggles, board-mounted, bushing through PCB void</t>
+          <t>Dedicated LED power only (VBUS+GND+CC). No data lines.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SWD header 1x3</t>
+          <t>Tactile button</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>J5</t>
+          <t>SW1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1x3 2.54mm</t>
+          <t>SMD tactile 4P</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -867,12 +867,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>header 1x3</t>
+          <t>tactile 3x4mm</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Debug/reflash (optional). Can be pads only.</t>
+          <t>SW1=BOOTSEL, SW2=RUN/reset.</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SW1;SW2</t>
+          <t>SW2</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>D1;D2;D3;D4;D5;D6;D7;D8;D9;D10;D11;D12;D13;D14;D15;D16;D17;D18;D19;D20;D21;D22;D23;D24;D25;D26;D27;D28</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -943,254 +943,2142 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>5.1k</t>
+          <t>LED red 1206</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>R1;R2;R3;R4</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>R0402</t>
+          <t>LED-1206</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>5.1k 0402</t>
+          <t>red 1206 diffused</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>USB-C CC pulldowns: 2 per connector (J1,J2).</t>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>LED red 1206</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>R5;R6</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>R0402</t>
+          <t>LED-1206</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>27R 0402</t>
+          <t>red 1206 diffused</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>USB D+/D- series resistors (J1 data only).</t>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2.4k</t>
+          <t>LED red 1206</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>R7;R8</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>R0402</t>
+          <t>LED-1206</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.4k 0402</t>
+          <t>red 1206 diffused</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>TLC5947 IREF (sets per-LED current ~15mA; raise R to lower current/heat).</t>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>LED red 1206</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>R9;R10;R11;R12;R13;R14;R15;R16;R17;R18</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>R0402</t>
+          <t>LED-1206</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10k 0402</t>
+          <t>red 1206 diffused</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Pull-ups: SD CS+data (4), command-switch inputs (4), spares (2).</t>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>100nF</t>
+          <t>LED red 1206</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>C1;C2;C3;C4;C5;C6;C7;C8;C9;C10;C11;C12;C13;C14;C15</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>C0402</t>
+          <t>LED-1206</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>100nF 0402</t>
+          <t>red 1206 diffused</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1uF</t>
+          <t>LED red 1206</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>C16;C17;C18;C19</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>C0402</t>
+          <t>LED-1206</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1uF 0402</t>
+          <t>red 1206 diffused</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>RP2040 core (1.1V) decoupling + SD socket local.</t>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>10uF</t>
+          <t>LED red 1206</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>C20;C21;C22</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>C0805</t>
+          <t>LED-1206</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>10uF 0805</t>
+          <t>red 1206 diffused</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Bulk on 3.3V logic, LED rail, and USB VBUS.</t>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>D11</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>D14</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>D15</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>D16</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>D17</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>D18</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>D19</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>D21</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>D22</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>D24</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>D25</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>D26</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>D27</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>LED red 1206</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>D28</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>LED-1206</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>red 1206 diffused</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>5.1k</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>R0402</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>5.1k 0402</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>USB-C CC pulldowns: 2 per connector (J1,J2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>5.1k</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>R0402</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>5.1k 0402</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>USB-C CC pulldowns: 2 per connector (J1,J2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>5.1k</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>R0402</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>5.1k 0402</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>USB-C CC pulldowns: 2 per connector (J1,J2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>5.1k</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>R0402</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>5.1k 0402</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>USB-C CC pulldowns: 2 per connector (J1,J2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>R0402</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>27R 0402</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>USB D+/D- series resistors (J1 data only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>R0402</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>27R 0402</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>USB D+/D- series resistors (J1 data only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2.4k</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>R7</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>R0402</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2.4k 0402</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>TLC5947 IREF (sets per-LED current ~15mA; raise R to lower current/heat).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2.4k</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>R8</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>R0402</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2.4k 0402</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>TLC5947 IREF (sets per-LED current ~15mA; raise R to lower current/heat).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>10k</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>R9</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>R0402</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>10k 0402</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Pull-ups: SD CS+data (4), command-switch inputs (4), spares (2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>10k</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>R10</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>R0402</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>10k 0402</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Pull-ups: SD CS+data (4), command-switch inputs (4), spares (2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>10k</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>R11</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>R0402</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>10k 0402</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Pull-ups: SD CS+data (4), command-switch inputs (4), spares (2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>10k</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>R12</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>R0402</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>10k 0402</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Pull-ups: SD CS+data (4), command-switch inputs (4), spares (2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>10k</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>R13</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>R0402</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>10k 0402</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Pull-ups: SD CS+data (4), command-switch inputs (4), spares (2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>10k</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>R14</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>R0402</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>10k 0402</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Pull-ups: SD CS+data (4), command-switch inputs (4), spares (2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>10k</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>R15</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>R0402</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>10k 0402</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Pull-ups: SD CS+data (4), command-switch inputs (4), spares (2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>10k</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>R16</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>R0402</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>10k 0402</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Pull-ups: SD CS+data (4), command-switch inputs (4), spares (2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>100nF</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>100nF 0402</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>100nF</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>100nF 0402</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>100nF</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>100nF 0402</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>100nF</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>100nF 0402</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>100nF</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>100nF 0402</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>100nF</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>100nF 0402</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>100nF</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>100nF 0402</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>100nF</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>100nF 0402</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>100nF</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>100nF 0402</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>100nF</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>100nF 0402</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>100nF</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>C11</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>100nF 0402</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>100nF</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>C12</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>100nF 0402</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>100nF</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>100nF 0402</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>100nF</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>C14</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>100nF 0402</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>100nF</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>C15</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>100nF 0402</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>1uF</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>C16</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>1uF 0402</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>RP2040 core (1.1V) decoupling + SD socket local.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>1uF</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>1uF 0402</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>RP2040 core (1.1V) decoupling + SD socket local.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>1uF</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>C18</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>1uF 0402</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>RP2040 core (1.1V) decoupling + SD socket local.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>1uF</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>C19</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>1uF 0402</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>RP2040 core (1.1V) decoupling + SD socket local.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>10uF</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>C20</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>C0805</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>10uF 0805</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Bulk on 3.3V logic, LED rail, and USB VBUS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>10uF</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>C21</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>C0805</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>10uF 0805</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Bulk on 3.3V logic, LED rail, and USB VBUS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>10uF</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>C22</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>C0805</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>10uF 0805</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Bulk on 3.3V logic, LED rail, and USB VBUS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
           <t>15pF</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>C23;C24</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>C23</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
         <is>
           <t>C0402</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
         <is>
           <t>15pF 0402</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Crystal load caps (tune to crystal spec).</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>15pF</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>C24</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>C0402</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>15pF 0402</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
         <is>
           <t>Crystal load caps (tune to crystal spec).</t>
         </is>

</xml_diff>

<commit_message>
fab(rev5): fab-assembled through-hole toggles in BOM+CPL+XYRS
User wants the fab house to assemble the 12 toggles. Added to BOTH vendor
packages (BOM<->CPL / BOM<->XYRS verified 1:1 at 94 rows each):
  SWD0-7  MTS-102 latching  @ void centers (49.325..154.325, 156.825)
  SWC0-3  MTS-103-M momentary @ (182.325..227.325, 156.825)
All: Top side (pads are F.Cu), rotation 0 (terminals toward LED rows),
placement = bushing center = board-void center (measured Edge.Cuts).
Still user-fitted: R17/R18 spares, J5 optional header (not in CPL/XYRS).
jlcpcb-cpl/ copy, both BOMs (csv+xlsx), both zips, README updated.
</commit_message>
<xml_diff>
--- a/hardware/fab-rev5/imspi8080-rev5-bom.xlsx
+++ b/hardware/fab-rev5/imspi8080-rev5-bom.xlsx
@@ -417,15 +417,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F83"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="5" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3084,6 +3084,390 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Mini-toggle SPDT ON-ON (latching)</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>SWD0</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>MTS-102</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>MTS-102</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>TH, bushing through board void; terminals solder to SWD0V/S/G pads (F.Cu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Mini-toggle SPDT ON-ON (latching)</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>SWD1</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>MTS-102</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>MTS-102</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>TH, bushing through board void; terminals solder to SWD1V/S/G pads (F.Cu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Mini-toggle SPDT ON-ON (latching)</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>SWD2</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>MTS-102</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>MTS-102</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>TH, bushing through board void; terminals solder to SWD2V/S/G pads (F.Cu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Mini-toggle SPDT ON-ON (latching)</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>SWD3</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>MTS-102</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>MTS-102</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>TH, bushing through board void; terminals solder to SWD3V/S/G pads (F.Cu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Mini-toggle SPDT ON-ON (latching)</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>SWD4</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>MTS-102</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>MTS-102</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>TH, bushing through board void; terminals solder to SWD4V/S/G pads (F.Cu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Mini-toggle SPDT ON-ON (latching)</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>SWD5</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>MTS-102</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>MTS-102</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>TH, bushing through board void; terminals solder to SWD5V/S/G pads (F.Cu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Mini-toggle SPDT ON-ON (latching)</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>SWD6</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>MTS-102</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>MTS-102</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>TH, bushing through board void; terminals solder to SWD6V/S/G pads (F.Cu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Mini-toggle SPDT ON-ON (latching)</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>SWD7</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>MTS-102</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>MTS-102</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>TH, bushing through board void; terminals solder to SWD7V/S/G pads (F.Cu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Mini-toggle SPDT momentary</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>SWC0</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>MTS-103-M</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>MTS-103-M</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>TH, bushing through board void; terminals solder to SWC0V/C/G pads (F.Cu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Mini-toggle SPDT momentary</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>SWC1</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>MTS-103-M</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>MTS-103-M</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>TH, bushing through board void; terminals solder to SWC1V/C/G pads (F.Cu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Mini-toggle SPDT momentary</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>SWC2</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>MTS-103-M</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>MTS-103-M</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>TH, bushing through board void; terminals solder to SWC2V/C/G pads (F.Cu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Mini-toggle SPDT momentary</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>SWC3</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>MTS-103-M</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>MTS-103-M</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>TH, bushing through board void; terminals solder to SWC3V/C/G pads (F.Cu)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fab(rev5): add J5 debug header to assembly data (both vendors)
J5 1x3 2.54mm TH header now in BOM+CPL (JLCPCB) and BOM+XYRS (MacroFab):
position (203.375, 98.875) rot 0 Top from the board footprint (pads
N$1/N$2/GND). Verified 1:1 at 95 rows per vendor. Only R17/R18 spares
remain user-fitted. Zips + README refreshed.
</commit_message>
<xml_diff>
--- a/hardware/fab-rev5/imspi8080-rev5-bom.xlsx
+++ b/hardware/fab-rev5/imspi8080-rev5-bom.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -3468,6 +3468,38 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>SWD header 1x3</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>J5</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>1x3 2.54mm</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>header 1x3</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Debug/reflash (optional). Through-hole 2.54mm header, top side.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fab(rev5): LCSC part numbers in BOM for JLCPCB auto-match
Adds 'LCSC Part #' column (22 rows) so the JLCPCB matcher resolves the
parts it couldn't find: RP2040 C2761095, flash C97521, TLC5947 C1554203,
165 C43420, USB-C C165948, crystal C9002, microSD C91145 (verify package),
MTS-102=C1788492, MT-0-103 C1788493 (VERIFY momentary in datasheet; note
says supply MTS-103-M yourself if latching-only). SW1/SW2/J5 annotated as
tool-picked. Passives/LEDs stay blank (JLCPCB auto-matches them).
</commit_message>
<xml_diff>
--- a/hardware/fab-rev5/imspi8080-rev5-bom.xlsx
+++ b/hardware/fab-rev5/imspi8080-rev5-bom.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F96"/>
+  <dimension ref="A1:G96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -426,6 +426,7 @@
     <col width="5" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -459,6 +460,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>LCSC Part #</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -491,6 +497,11 @@
           <t>MCU. Copy RP2040 minimal reference design. Extended part.</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>C2761095</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -523,6 +534,11 @@
           <t>Boot flash (firmware lives here). Basic/common.</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>C97521</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -555,6 +571,11 @@
           <t>Core clock. Basic. Load caps C_Y1a/b.</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>C9002</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -587,6 +608,11 @@
           <t>LED drivers, daisy-chained. Extended part (1 line = both).</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>C1554203</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -619,6 +645,11 @@
           <t>LED drivers, daisy-chained. Extended part (1 line = both).</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>C1554203</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -651,6 +682,11 @@
           <t>Switch inputs, daisy-chained.</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>C43420</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -683,6 +719,11 @@
           <t>Switch inputs, daisy-chained.</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>C43420</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -712,7 +753,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Data storage (optional). Pick a JLCPCB-library SMD socket.</t>
+          <t>Data storage (optional). Pick a JLCPCB-library SMD socket. | LCSC C91145: VERIFY package outline vs footprint before confirming</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>C91145</t>
         </is>
       </c>
     </row>
@@ -747,6 +793,7 @@
           <t>3.3V logic rail from USB-C #1 VBUS. Basic.</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -779,6 +826,7 @@
           <t>3.3V LED anode rail from USB-C #2 VBUS (keeps drivers cool).</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -811,6 +859,11 @@
           <t>Power + data to the Pi. 2x CC resistors + 2x D series R.</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>C165948</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -843,6 +896,11 @@
           <t>Dedicated LED power only (VBUS+GND+CC). No data lines.</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>C165948</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -872,9 +930,10 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>SW1=BOOTSEL, SW2=RUN/reset.</t>
-        </is>
-      </c>
+          <t>SW1=BOOTSEL, SW2=RUN/reset. | pick any in-stock 3x4mm SMD tactile in the JLCPCB tool</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -904,9 +963,10 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>SW1=BOOTSEL, SW2=RUN/reset.</t>
-        </is>
-      </c>
+          <t>SW1=BOOTSEL, SW2=RUN/reset. | pick any in-stock 3x4mm SMD tactile in the JLCPCB tool</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -939,6 +999,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -971,6 +1032,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1003,6 +1065,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1035,6 +1098,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1067,6 +1131,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1099,6 +1164,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1131,6 +1197,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1163,6 +1230,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1195,6 +1263,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1227,6 +1296,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1259,6 +1329,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1291,6 +1362,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1323,6 +1395,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1355,6 +1428,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1387,6 +1461,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1419,6 +1494,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1451,6 +1527,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1483,6 +1560,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1515,6 +1593,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1547,6 +1626,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1579,6 +1659,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1611,6 +1692,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1643,6 +1725,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1675,6 +1758,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1707,6 +1791,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1739,6 +1824,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1771,6 +1857,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1803,6 +1890,7 @@
           <t>No series resistors (TLC5947 is constant-current). Check PCBA type is not Standard-Only if you want Economic.</t>
         </is>
       </c>
+      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1835,6 +1923,7 @@
           <t>USB-C CC pulldowns: 2 per connector (J1,J2).</t>
         </is>
       </c>
+      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1867,6 +1956,7 @@
           <t>USB-C CC pulldowns: 2 per connector (J1,J2).</t>
         </is>
       </c>
+      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1899,6 +1989,7 @@
           <t>USB-C CC pulldowns: 2 per connector (J1,J2).</t>
         </is>
       </c>
+      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1931,6 +2022,7 @@
           <t>USB-C CC pulldowns: 2 per connector (J1,J2).</t>
         </is>
       </c>
+      <c r="G47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1963,6 +2055,7 @@
           <t>USB D+/D- series resistors (J1 data only).</t>
         </is>
       </c>
+      <c r="G48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1995,6 +2088,7 @@
           <t>USB D+/D- series resistors (J1 data only).</t>
         </is>
       </c>
+      <c r="G49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2027,6 +2121,7 @@
           <t>TLC5947 IREF (sets per-LED current ~15mA; raise R to lower current/heat).</t>
         </is>
       </c>
+      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2059,6 +2154,7 @@
           <t>TLC5947 IREF (sets per-LED current ~15mA; raise R to lower current/heat).</t>
         </is>
       </c>
+      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2091,6 +2187,7 @@
           <t>Pull-ups: SD CS+data (4), command-switch inputs (4), spares (2).</t>
         </is>
       </c>
+      <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2123,6 +2220,7 @@
           <t>Pull-ups: SD CS+data (4), command-switch inputs (4), spares (2).</t>
         </is>
       </c>
+      <c r="G53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2155,6 +2253,7 @@
           <t>Pull-ups: SD CS+data (4), command-switch inputs (4), spares (2).</t>
         </is>
       </c>
+      <c r="G54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2187,6 +2286,7 @@
           <t>Pull-ups: SD CS+data (4), command-switch inputs (4), spares (2).</t>
         </is>
       </c>
+      <c r="G55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2219,6 +2319,7 @@
           <t>Pull-ups: SD CS+data (4), command-switch inputs (4), spares (2).</t>
         </is>
       </c>
+      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2251,6 +2352,7 @@
           <t>Pull-ups: SD CS+data (4), command-switch inputs (4), spares (2).</t>
         </is>
       </c>
+      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2283,6 +2385,7 @@
           <t>Pull-ups: SD CS+data (4), command-switch inputs (4), spares (2).</t>
         </is>
       </c>
+      <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2315,6 +2418,7 @@
           <t>Pull-ups: SD CS+data (4), command-switch inputs (4), spares (2).</t>
         </is>
       </c>
+      <c r="G59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2347,6 +2451,7 @@
           <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
         </is>
       </c>
+      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2379,6 +2484,7 @@
           <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
         </is>
       </c>
+      <c r="G61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2411,6 +2517,7 @@
           <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
         </is>
       </c>
+      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2443,6 +2550,7 @@
           <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
         </is>
       </c>
+      <c r="G63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2475,6 +2583,7 @@
           <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
         </is>
       </c>
+      <c r="G64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2507,6 +2616,7 @@
           <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
         </is>
       </c>
+      <c r="G65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2539,6 +2649,7 @@
           <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
         </is>
       </c>
+      <c r="G66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2571,6 +2682,7 @@
           <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
         </is>
       </c>
+      <c r="G67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2603,6 +2715,7 @@
           <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
         </is>
       </c>
+      <c r="G68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2635,6 +2748,7 @@
           <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
         </is>
       </c>
+      <c r="G69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2667,6 +2781,7 @@
           <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
         </is>
       </c>
+      <c r="G70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2699,6 +2814,7 @@
           <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
         </is>
       </c>
+      <c r="G71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2731,6 +2847,7 @@
           <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
         </is>
       </c>
+      <c r="G72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2763,6 +2880,7 @@
           <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
         </is>
       </c>
+      <c r="G73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2795,6 +2913,7 @@
           <t>Per-IC decoupling (RP2040 needs several, TLC5947 x2, 165 x2, flash, SD, regs).</t>
         </is>
       </c>
+      <c r="G74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2827,6 +2946,7 @@
           <t>RP2040 core (1.1V) decoupling + SD socket local.</t>
         </is>
       </c>
+      <c r="G75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2859,6 +2979,7 @@
           <t>RP2040 core (1.1V) decoupling + SD socket local.</t>
         </is>
       </c>
+      <c r="G76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2891,6 +3012,7 @@
           <t>RP2040 core (1.1V) decoupling + SD socket local.</t>
         </is>
       </c>
+      <c r="G77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2923,6 +3045,7 @@
           <t>RP2040 core (1.1V) decoupling + SD socket local.</t>
         </is>
       </c>
+      <c r="G78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2955,6 +3078,7 @@
           <t>Bulk on 3.3V logic, LED rail, and USB VBUS.</t>
         </is>
       </c>
+      <c r="G79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2987,6 +3111,7 @@
           <t>Bulk on 3.3V logic, LED rail, and USB VBUS.</t>
         </is>
       </c>
+      <c r="G80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3019,6 +3144,7 @@
           <t>Bulk on 3.3V logic, LED rail, and USB VBUS.</t>
         </is>
       </c>
+      <c r="G81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3051,6 +3177,7 @@
           <t>Crystal load caps (tune to crystal spec).</t>
         </is>
       </c>
+      <c r="G82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3083,6 +3210,7 @@
           <t>Crystal load caps (tune to crystal spec).</t>
         </is>
       </c>
+      <c r="G83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3115,6 +3243,11 @@
           <t>TH, bushing through board void; terminals solder to SWD0V/S/G pads (F.Cu)</t>
         </is>
       </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>C1788492</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3147,6 +3280,11 @@
           <t>TH, bushing through board void; terminals solder to SWD1V/S/G pads (F.Cu)</t>
         </is>
       </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>C1788492</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3179,6 +3317,11 @@
           <t>TH, bushing through board void; terminals solder to SWD2V/S/G pads (F.Cu)</t>
         </is>
       </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>C1788492</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3211,6 +3354,11 @@
           <t>TH, bushing through board void; terminals solder to SWD3V/S/G pads (F.Cu)</t>
         </is>
       </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>C1788492</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3243,6 +3391,11 @@
           <t>TH, bushing through board void; terminals solder to SWD4V/S/G pads (F.Cu)</t>
         </is>
       </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>C1788492</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3275,6 +3428,11 @@
           <t>TH, bushing through board void; terminals solder to SWD5V/S/G pads (F.Cu)</t>
         </is>
       </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>C1788492</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3307,6 +3465,11 @@
           <t>TH, bushing through board void; terminals solder to SWD6V/S/G pads (F.Cu)</t>
         </is>
       </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>C1788492</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3339,6 +3502,11 @@
           <t>TH, bushing through board void; terminals solder to SWD7V/S/G pads (F.Cu)</t>
         </is>
       </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>C1788492</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3368,7 +3536,12 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>TH, bushing through board void; terminals solder to SWC0V/C/G pads (F.Cu)</t>
+          <t>TH, bushing through board void; terminals solder to SWC0V/C/G pads (F.Cu) | LCSC C1788493: VERIFY momentary (ON)-OFF-(ON) in datasheet; if latching-only, supply MTS-103-M yourself</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>C1788493</t>
         </is>
       </c>
     </row>
@@ -3400,7 +3573,12 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>TH, bushing through board void; terminals solder to SWC1V/C/G pads (F.Cu)</t>
+          <t>TH, bushing through board void; terminals solder to SWC1V/C/G pads (F.Cu) | LCSC C1788493: VERIFY momentary (ON)-OFF-(ON) in datasheet; if latching-only, supply MTS-103-M yourself</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>C1788493</t>
         </is>
       </c>
     </row>
@@ -3432,7 +3610,12 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>TH, bushing through board void; terminals solder to SWC2V/C/G pads (F.Cu)</t>
+          <t>TH, bushing through board void; terminals solder to SWC2V/C/G pads (F.Cu) | LCSC C1788493: VERIFY momentary (ON)-OFF-(ON) in datasheet; if latching-only, supply MTS-103-M yourself</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>C1788493</t>
         </is>
       </c>
     </row>
@@ -3464,7 +3647,12 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>TH, bushing through board void; terminals solder to SWC3V/C/G pads (F.Cu)</t>
+          <t>TH, bushing through board void; terminals solder to SWC3V/C/G pads (F.Cu) | LCSC C1788493: VERIFY momentary (ON)-OFF-(ON) in datasheet; if latching-only, supply MTS-103-M yourself</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>C1788493</t>
         </is>
       </c>
     </row>
@@ -3496,9 +3684,10 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Debug/reflash (optional). Through-hole 2.54mm header, top side.</t>
-        </is>
-      </c>
+          <t>Debug/reflash (optional). Through-hole 2.54mm header, top side. | pick any 2.54mm 1x3 TH header in the JLCPCB tool</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>